<commit_message>
fix(about-us): group contributor XFs into 2 grids (Our Contributors + WKND Guides)
The parser emitted one contributors block per person (7 stacked blocks). Group
the person XFs by their preceding section H2 so it emits ONE grid per section:
Our Contributors (4) and WKND Guides (3), matching the source layout.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -11,17 +11,23 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="162">
   <si>
     <t>_reportFile</t>
   </si>
   <si>
+    <t>author</t>
+  </si>
+  <si>
     <t>blocks</t>
   </si>
   <si>
     <t>path</t>
   </si>
   <si>
+    <t>publicationDate</t>
+  </si>
+  <si>
     <t>status</t>
   </si>
   <si>
@@ -40,7 +46,10 @@
     <t>us/en.report.json</t>
   </si>
   <si>
-    <t>["carousel-hero","columns-featured","columns-featured","cards-teaser","cards-teaser","hero-promo","hero-promo"]</t>
+    <t/>
+  </si>
+  <si>
+    <t>["carousel-hero","columns-featured","columns-featured","article-list","article-list","hero-promo","hero-promo"]</t>
   </si>
   <si>
     <t>us/en</t>
@@ -52,7 +61,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-08-06T08:09:21.761Z</t>
+    <t>2026-08-06T19:05:35.144Z</t>
   </si>
   <si>
     <t>WKND Adventures and Travel</t>
@@ -73,7 +82,7 @@
     <t>about-us</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:03.070Z</t>
+    <t>2026-08-06T19:17:25.706Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -82,6 +91,48 @@
     <t>https://wknd.site/us/en/about-us.html</t>
   </si>
   <si>
+    <t>us/en/adventures.report.json</t>
+  </si>
+  <si>
+    <t>["hero-intro","hero-intro","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures</t>
+  </si>
+  <si>
+    <t>adventure-listing</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:10:07.880Z</t>
+  </si>
+  <si>
+    <t>Adventures</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures.html</t>
+  </si>
+  <si>
+    <t>us/en/faqs.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-faq"]</t>
+  </si>
+  <si>
+    <t>us/en/faqs</t>
+  </si>
+  <si>
+    <t>faq-page</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:10:12.791Z</t>
+  </si>
+  <si>
+    <t>FAQs</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/faqs.html</t>
+  </si>
+  <si>
     <t>us/en/magazine.report.json</t>
   </si>
   <si>
@@ -101,6 +152,351 @@
   </si>
   <si>
     <t>https://wknd.site/us/en/magazine.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp.report.json</t>
+  </si>
+  <si>
+    <t>["carousel-gallery","adventure-details","adventure-details","tabs-adventure"]</t>
+  </si>
+  <si>
+    <t>us/en/adventures/bali-surf-camp</t>
+  </si>
+  <si>
+    <t>adventure-detail</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:10:47.301Z</t>
+  </si>
+  <si>
+    <t>Bali Surf Camp</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/bali-surf-camp.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/beervana-portland</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:10:53.657Z</t>
+  </si>
+  <si>
+    <t>Beervana in Portland</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/beervana-portland.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/climbing-new-zealand</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:10:59.799Z</t>
+  </si>
+  <si>
+    <t>Climbing New Zealand</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/climbing-new-zealand.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/colorado-rock-climbing</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:05.230Z</t>
+  </si>
+  <si>
+    <t>Colorado Rock Climbing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/colorado-rock-climbing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-southern-utah</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:10.049Z</t>
+  </si>
+  <si>
+    <t>Cycling Southern Utah</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-southern-utah.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/cycling-tuscany</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:14.793Z</t>
+  </si>
+  <si>
+    <t>Cycling Tuscany</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/cycling-tuscany.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/downhill-skiing-wyoming</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:21.514Z</t>
+  </si>
+  <si>
+    <t>Downhill Skiing Wyoming</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/downhill-skiing-wyoming.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/gastronomic-marais-tour</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:27.625Z</t>
+  </si>
+  <si>
+    <t>Gastronomic Marais Tour</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/gastronomic-marais-tour.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/napa-wine-tasting</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:33.534Z</t>
+  </si>
+  <si>
+    <t>Napa Wine Tasting</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/napa-wine-tasting.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/riverside-camping-australia</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:38.037Z</t>
+  </si>
+  <si>
+    <t>Riverside Camping</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/riverside-camping-australia.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/ski-touring-mont-blanc</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:42.932Z</t>
+  </si>
+  <si>
+    <t>Ski Touring Mont Blanc</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/ski-touring-mont-blanc.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/surf-camp-costa-rica</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:48.059Z</t>
+  </si>
+  <si>
+    <t>Surf Camp in Costa Rica</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/surf-camp-costa-rica.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/tahoe-skiing</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:52.326Z</t>
+  </si>
+  <si>
+    <t>Tahoe Skiing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/tahoe-skiing.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/west-coast-cycling</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:11:57.335Z</t>
+  </si>
+  <si>
+    <t>West Coast Cycling</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/west-coast-cycling.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/whistler-mountain-biking</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:12:03.133Z</t>
+  </si>
+  <si>
+    <t>Whistler Mountain Biking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/whistler-mountain-biking.html</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking.report.json</t>
+  </si>
+  <si>
+    <t>us/en/adventures/yosemite-backpacking</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:12:08.188Z</t>
+  </si>
+  <si>
+    <t>Yosemite Backpacking</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/adventures/yosemite-backpacking.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing.report.json</t>
+  </si>
+  <si>
+    <t>Jacob Wester</t>
+  </si>
+  <si>
+    <t>["article-author","cards-related"]</t>
+  </si>
+  <si>
+    <t>us/en/magazine/arctic-surfing</t>
+  </si>
+  <si>
+    <t>2020-07-09</t>
+  </si>
+  <si>
+    <t>magazine-article</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:25:31.199Z</t>
+  </si>
+  <si>
+    <t>Arctic Surfing</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/arctic-surfing.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks.report.json</t>
+  </si>
+  <si>
+    <t>Stacey Roswells</t>
+  </si>
+  <si>
+    <t>us/en/magazine/guide-la-skateparks</t>
+  </si>
+  <si>
+    <t>2020-09-30</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:25:35.320Z</t>
+  </si>
+  <si>
+    <t>Ultimate Guide to LA Skateparks</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/guide-la-skateparks.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf.report.json</t>
+  </si>
+  <si>
+    <t>Justin Barr</t>
+  </si>
+  <si>
+    <t>us/en/magazine/san-diego-surf</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:25:39.721Z</t>
+  </si>
+  <si>
+    <t>San Diego Surf Spots</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/san-diego-surf.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring.report.json</t>
+  </si>
+  <si>
+    <t>Sofia Sjöberg</t>
+  </si>
+  <si>
+    <t>us/en/magazine/ski-touring</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:25:43.664Z</t>
+  </si>
+  <si>
+    <t>Ski Touring</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/ski-touring.html</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia.report.json</t>
+  </si>
+  <si>
+    <t>us/en/magazine/western-australia</t>
+  </si>
+  <si>
+    <t>2026-08-06T08:25:49.650Z</t>
+  </si>
+  <si>
+    <t>Western Australia</t>
+  </si>
+  <si>
+    <t>https://wknd.site/us/en/magazine/western-australia.html</t>
   </si>
 </sst>
 </file>
@@ -489,19 +885,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="28" customWidth="1"/>
-    <col min="8" max="8" width="39" customWidth="1"/>
+    <col min="1" max="1" width="50" customWidth="1"/>
+    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="46" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
+    <col min="7" max="7" width="19" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="33" customWidth="1"/>
+    <col min="10" max="10" width="50" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -526,87 +924,847 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H4" t="s">
-        <v>29</v>
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" t="s">
+        <v>44</v>
+      </c>
+      <c r="I6" t="s">
+        <v>45</v>
+      </c>
+      <c r="J6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J7" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>50</v>
+      </c>
+      <c r="H8" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" t="s">
+        <v>61</v>
+      </c>
+      <c r="I9" t="s">
+        <v>62</v>
+      </c>
+      <c r="J9" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" t="s">
+        <v>65</v>
+      </c>
+      <c r="E10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>50</v>
+      </c>
+      <c r="H10" t="s">
+        <v>66</v>
+      </c>
+      <c r="I10" t="s">
+        <v>67</v>
+      </c>
+      <c r="J10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>69</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" t="s">
+        <v>70</v>
+      </c>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" t="s">
+        <v>14</v>
+      </c>
+      <c r="G11" t="s">
+        <v>50</v>
+      </c>
+      <c r="H11" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" t="s">
+        <v>72</v>
+      </c>
+      <c r="J11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" t="s">
+        <v>75</v>
+      </c>
+      <c r="E12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" t="s">
+        <v>76</v>
+      </c>
+      <c r="I12" t="s">
+        <v>77</v>
+      </c>
+      <c r="J12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" t="s">
+        <v>80</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>50</v>
+      </c>
+      <c r="H13" t="s">
+        <v>81</v>
+      </c>
+      <c r="I13" t="s">
+        <v>82</v>
+      </c>
+      <c r="J13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" t="s">
+        <v>85</v>
+      </c>
+      <c r="E14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>50</v>
+      </c>
+      <c r="H14" t="s">
+        <v>86</v>
+      </c>
+      <c r="I14" t="s">
+        <v>87</v>
+      </c>
+      <c r="J14" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" t="s">
+        <v>90</v>
+      </c>
+      <c r="E15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" t="s">
+        <v>91</v>
+      </c>
+      <c r="I15" t="s">
+        <v>92</v>
+      </c>
+      <c r="J15" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>94</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
+        <v>95</v>
+      </c>
+      <c r="E16" t="s">
+        <v>11</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>50</v>
+      </c>
+      <c r="H16" t="s">
+        <v>96</v>
+      </c>
+      <c r="I16" t="s">
+        <v>97</v>
+      </c>
+      <c r="J16" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" t="s">
+        <v>100</v>
+      </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>50</v>
+      </c>
+      <c r="H17" t="s">
+        <v>101</v>
+      </c>
+      <c r="I17" t="s">
+        <v>102</v>
+      </c>
+      <c r="J17" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" t="s">
+        <v>105</v>
+      </c>
+      <c r="E18" t="s">
+        <v>11</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>50</v>
+      </c>
+      <c r="H18" t="s">
+        <v>106</v>
+      </c>
+      <c r="I18" t="s">
+        <v>107</v>
+      </c>
+      <c r="J18" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>109</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" t="s">
+        <v>110</v>
+      </c>
+      <c r="E19" t="s">
+        <v>11</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>50</v>
+      </c>
+      <c r="H19" t="s">
+        <v>111</v>
+      </c>
+      <c r="I19" t="s">
+        <v>112</v>
+      </c>
+      <c r="J19" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>114</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" t="s">
+        <v>115</v>
+      </c>
+      <c r="E20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>50</v>
+      </c>
+      <c r="H20" t="s">
+        <v>116</v>
+      </c>
+      <c r="I20" t="s">
+        <v>117</v>
+      </c>
+      <c r="J20" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E21" t="s">
+        <v>11</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>50</v>
+      </c>
+      <c r="H21" t="s">
+        <v>121</v>
+      </c>
+      <c r="I21" t="s">
+        <v>122</v>
+      </c>
+      <c r="J21" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>124</v>
+      </c>
+      <c r="B22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" t="s">
+        <v>125</v>
+      </c>
+      <c r="E22" t="s">
+        <v>11</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>50</v>
+      </c>
+      <c r="H22" t="s">
+        <v>126</v>
+      </c>
+      <c r="I22" t="s">
+        <v>127</v>
+      </c>
+      <c r="J22" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>129</v>
+      </c>
+      <c r="B23" t="s">
+        <v>130</v>
+      </c>
+      <c r="C23" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" t="s">
+        <v>132</v>
+      </c>
+      <c r="E23" t="s">
+        <v>133</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>134</v>
+      </c>
+      <c r="H23" t="s">
+        <v>135</v>
+      </c>
+      <c r="I23" t="s">
+        <v>136</v>
+      </c>
+      <c r="J23" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>138</v>
+      </c>
+      <c r="B24" t="s">
+        <v>139</v>
+      </c>
+      <c r="C24" t="s">
+        <v>131</v>
+      </c>
+      <c r="D24" t="s">
+        <v>140</v>
+      </c>
+      <c r="E24" t="s">
+        <v>141</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>134</v>
+      </c>
+      <c r="H24" t="s">
+        <v>142</v>
+      </c>
+      <c r="I24" t="s">
+        <v>143</v>
+      </c>
+      <c r="J24" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>145</v>
+      </c>
+      <c r="B25" t="s">
+        <v>146</v>
+      </c>
+      <c r="C25" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" t="s">
+        <v>147</v>
+      </c>
+      <c r="E25" t="s">
+        <v>141</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>134</v>
+      </c>
+      <c r="H25" t="s">
+        <v>148</v>
+      </c>
+      <c r="I25" t="s">
+        <v>149</v>
+      </c>
+      <c r="J25" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>151</v>
+      </c>
+      <c r="B26" t="s">
+        <v>152</v>
+      </c>
+      <c r="C26" t="s">
+        <v>131</v>
+      </c>
+      <c r="D26" t="s">
+        <v>153</v>
+      </c>
+      <c r="E26" t="s">
+        <v>141</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>134</v>
+      </c>
+      <c r="H26" t="s">
+        <v>154</v>
+      </c>
+      <c r="I26" t="s">
+        <v>155</v>
+      </c>
+      <c r="J26" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>157</v>
+      </c>
+      <c r="B27" t="s">
+        <v>152</v>
+      </c>
+      <c r="C27" t="s">
+        <v>131</v>
+      </c>
+      <c r="D27" t="s">
+        <v>158</v>
+      </c>
+      <c r="E27" t="s">
+        <v>141</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>134</v>
+      </c>
+      <c r="H27" t="s">
+        <v>159</v>
+      </c>
+      <c r="I27" t="s">
+        <v>160</v>
+      </c>
+      <c r="J27" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:J1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: add migration.html analysis dashboard
Self-contained static migration-analysis page (served at /migration.html),
mirroring the capstone reference. Three tabs — Analysis, Migration Plan, Page
Inventory — tailored to this project: 28 URLs across 7 templates, the actual
query-index-driven listings, and the base+variant block consolidation
(carousel/hero/columns/cards/accordion/tabs) with article-list/contributors
kept as query-index blocks. Interactive inventory filter over the real
/us/en URL set.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-about-us.report.xlsx
+++ b/tools/importer/reports/import-about-us.report.xlsx
@@ -82,7 +82,7 @@
     <t>about-us</t>
   </si>
   <si>
-    <t>2026-08-06T19:17:25.706Z</t>
+    <t>2026-08-08T05:08:50.164Z</t>
   </si>
   <si>
     <t>About Us</t>
@@ -94,7 +94,7 @@
     <t>us/en/adventures.report.json</t>
   </si>
   <si>
-    <t>["hero-intro","hero-intro","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser","cards-teaser"]</t>
+    <t>["hero-promo","hero-promo","article-list"]</t>
   </si>
   <si>
     <t>us/en/adventures</t>
@@ -103,7 +103,7 @@
     <t>adventure-listing</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:07.880Z</t>
+    <t>2026-08-07T03:09:28.549Z</t>
   </si>
   <si>
     <t>Adventures</t>
@@ -136,7 +136,7 @@
     <t>us/en/magazine.report.json</t>
   </si>
   <si>
-    <t>["columns-featured","columns-featured","article-list","cards-teaser","cards-teaser"]</t>
+    <t>["columns-featured","columns-featured","article-list","article-list-members","article-list-members"]</t>
   </si>
   <si>
     <t>us/en/magazine</t>
@@ -145,7 +145,7 @@
     <t>magazine-landing</t>
   </si>
   <si>
-    <t>2026-08-06T08:09:58.122Z</t>
+    <t>2026-08-07T10:26:33.120Z</t>
   </si>
   <si>
     <t>Magazine</t>
@@ -166,7 +166,7 @@
     <t>adventure-detail</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:47.301Z</t>
+    <t>2026-08-07T03:52:36.551Z</t>
   </si>
   <si>
     <t>Bali Surf Camp</t>
@@ -181,7 +181,7 @@
     <t>us/en/adventures/beervana-portland</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:53.657Z</t>
+    <t>2026-08-07T03:52:41.602Z</t>
   </si>
   <si>
     <t>Beervana in Portland</t>
@@ -196,7 +196,7 @@
     <t>us/en/adventures/climbing-new-zealand</t>
   </si>
   <si>
-    <t>2026-08-06T08:10:59.799Z</t>
+    <t>2026-08-07T03:52:47.314Z</t>
   </si>
   <si>
     <t>Climbing New Zealand</t>
@@ -211,7 +211,7 @@
     <t>us/en/adventures/colorado-rock-climbing</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:05.230Z</t>
+    <t>2026-08-07T03:52:51.830Z</t>
   </si>
   <si>
     <t>Colorado Rock Climbing</t>
@@ -226,7 +226,7 @@
     <t>us/en/adventures/cycling-southern-utah</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:10.049Z</t>
+    <t>2026-08-07T03:52:56.771Z</t>
   </si>
   <si>
     <t>Cycling Southern Utah</t>
@@ -241,7 +241,7 @@
     <t>us/en/adventures/cycling-tuscany</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:14.793Z</t>
+    <t>2026-08-07T03:53:02.103Z</t>
   </si>
   <si>
     <t>Cycling Tuscany</t>
@@ -256,7 +256,7 @@
     <t>us/en/adventures/downhill-skiing-wyoming</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:21.514Z</t>
+    <t>2026-08-07T03:53:06.972Z</t>
   </si>
   <si>
     <t>Downhill Skiing Wyoming</t>
@@ -271,7 +271,7 @@
     <t>us/en/adventures/gastronomic-marais-tour</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:27.625Z</t>
+    <t>2026-08-07T03:53:11.981Z</t>
   </si>
   <si>
     <t>Gastronomic Marais Tour</t>
@@ -286,7 +286,7 @@
     <t>us/en/adventures/napa-wine-tasting</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:33.534Z</t>
+    <t>2026-08-07T03:53:16.988Z</t>
   </si>
   <si>
     <t>Napa Wine Tasting</t>
@@ -301,7 +301,7 @@
     <t>us/en/adventures/riverside-camping-australia</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:38.037Z</t>
+    <t>2026-08-07T03:53:21.395Z</t>
   </si>
   <si>
     <t>Riverside Camping</t>
@@ -316,7 +316,7 @@
     <t>us/en/adventures/ski-touring-mont-blanc</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:42.932Z</t>
+    <t>2026-08-07T03:53:25.566Z</t>
   </si>
   <si>
     <t>Ski Touring Mont Blanc</t>
@@ -331,7 +331,7 @@
     <t>us/en/adventures/surf-camp-costa-rica</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:48.059Z</t>
+    <t>2026-08-07T03:53:31.681Z</t>
   </si>
   <si>
     <t>Surf Camp in Costa Rica</t>
@@ -346,7 +346,7 @@
     <t>us/en/adventures/tahoe-skiing</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:52.326Z</t>
+    <t>2026-08-07T03:53:36.966Z</t>
   </si>
   <si>
     <t>Tahoe Skiing</t>
@@ -361,7 +361,7 @@
     <t>us/en/adventures/west-coast-cycling</t>
   </si>
   <si>
-    <t>2026-08-06T08:11:57.335Z</t>
+    <t>2026-08-07T03:53:40.930Z</t>
   </si>
   <si>
     <t>West Coast Cycling</t>
@@ -376,7 +376,7 @@
     <t>us/en/adventures/whistler-mountain-biking</t>
   </si>
   <si>
-    <t>2026-08-06T08:12:03.133Z</t>
+    <t>2026-08-07T03:53:46.408Z</t>
   </si>
   <si>
     <t>Whistler Mountain Biking</t>
@@ -391,7 +391,7 @@
     <t>us/en/adventures/yosemite-backpacking</t>
   </si>
   <si>
-    <t>2026-08-06T08:12:08.188Z</t>
+    <t>2026-08-07T03:53:52.237Z</t>
   </si>
   <si>
     <t>Yosemite Backpacking</t>
@@ -406,7 +406,7 @@
     <t>Jacob Wester</t>
   </si>
   <si>
-    <t>["article-author","cards-related"]</t>
+    <t>["article-author","article-list"]</t>
   </si>
   <si>
     <t>us/en/magazine/arctic-surfing</t>
@@ -418,7 +418,7 @@
     <t>magazine-article</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:31.199Z</t>
+    <t>2026-08-07T12:18:42.590Z</t>
   </si>
   <si>
     <t>Arctic Surfing</t>
@@ -439,7 +439,7 @@
     <t>2020-09-30</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:35.320Z</t>
+    <t>2026-08-07T12:18:48.179Z</t>
   </si>
   <si>
     <t>Ultimate Guide to LA Skateparks</t>
@@ -457,7 +457,7 @@
     <t>us/en/magazine/san-diego-surf</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:39.721Z</t>
+    <t>2026-08-07T12:18:53.759Z</t>
   </si>
   <si>
     <t>San Diego Surf Spots</t>
@@ -475,7 +475,7 @@
     <t>us/en/magazine/ski-touring</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:43.664Z</t>
+    <t>2026-08-07T12:18:58.899Z</t>
   </si>
   <si>
     <t>Ski Touring</t>
@@ -490,7 +490,7 @@
     <t>us/en/magazine/western-australia</t>
   </si>
   <si>
-    <t>2026-08-06T08:25:49.650Z</t>
+    <t>2026-08-07T12:19:04.623Z</t>
   </si>
   <si>
     <t>Western Australia</t>

</xml_diff>